<commit_message>
feat: enhance size-accuracy analysis with demanded curve overlay and update metrics
</commit_message>
<xml_diff>
--- a/RQ_experiments/RQ4/report/rq4_table.xlsx
+++ b/RQ_experiments/RQ4/report/rq4_table.xlsx
@@ -596,7 +596,7 @@
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K4" t="n">
         <v>2</v>
@@ -824,7 +824,7 @@
         <v>1051917.4</v>
       </c>
       <c r="H10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I10" t="n">
         <v>4</v>
@@ -947,7 +947,7 @@
         <v>5</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13" t="n">
         <v>3</v>
@@ -986,7 +986,7 @@
         <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
         <v>1</v>
@@ -1019,7 +1019,7 @@
         <v>1151983.32</v>
       </c>
       <c r="H15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I15" t="n">
         <v>4</v>
@@ -1064,7 +1064,7 @@
         <v>5</v>
       </c>
       <c r="J16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K16" t="n">
         <v>3</v>
@@ -1142,7 +1142,7 @@
         <v>4</v>
       </c>
       <c r="J18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K18" t="n">
         <v>1</v>
@@ -1370,13 +1370,13 @@
         <v>1276411.57</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
         <v>4</v>
       </c>
       <c r="J24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K24" t="n">
         <v>1</v>
@@ -1415,7 +1415,7 @@
         <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K25" t="n">
         <v>1</v>
@@ -1493,7 +1493,7 @@
         <v>3</v>
       </c>
       <c r="J27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K27" t="n">
         <v>1</v>
@@ -1727,7 +1727,7 @@
         <v>5</v>
       </c>
       <c r="J33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K33" t="n">
         <v>3</v>

</xml_diff>